<commit_message>
computational test results, visualisation, statistical testing, and pymoo fixes
</commit_message>
<xml_diff>
--- a/datasets.xlsx
+++ b/datasets.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erinfortin/Documents/Dissertation - Feature Selection/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erinfortin/Documents/Dissertation - Feature Selection/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0AB158-C211-F34D-BEAC-B7FE54F1F4AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D1BB1DC-72BF-6341-9851-301CBBDECD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="620" windowWidth="25580" windowHeight="28180" xr2:uid="{44673F34-DF5D-4845-98A3-3A36EA99668B}"/>
+    <workbookView xWindow="7480" yWindow="680" windowWidth="10020" windowHeight="17380" xr2:uid="{44673F34-DF5D-4845-98A3-3A36EA99668B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t>Name</t>
   </si>
@@ -56,34 +56,25 @@
     <t>isolet</t>
   </si>
   <si>
-    <t>breastcancer</t>
-  </si>
-  <si>
     <t>spambase</t>
   </si>
   <si>
     <t>lymphography</t>
   </si>
   <si>
-    <t>congressionalVR</t>
-  </si>
-  <si>
-    <t>communities-crime</t>
-  </si>
-  <si>
     <t>regression</t>
   </si>
   <si>
+    <t>bike-sharing</t>
+  </si>
+  <si>
+    <t>wave-energy</t>
+  </si>
+  <si>
+    <t>energy</t>
+  </si>
+  <si>
     <t>superconductivity</t>
-  </si>
-  <si>
-    <t>iot</t>
-  </si>
-  <si>
-    <t>bike-sharing</t>
-  </si>
-  <si>
-    <t>air-quality</t>
   </si>
 </sst>
 </file>
@@ -455,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00AA4E1-5793-AF45-B5C7-8B92B019128E}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -485,7 +476,7 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>17</v>
+        <v>94</v>
       </c>
       <c r="C3" t="s">
         <v>3</v>
@@ -496,7 +487,7 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>94</v>
+        <v>63</v>
       </c>
       <c r="C4" t="s">
         <v>3</v>
@@ -504,79 +495,35 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
         <v>7</v>
-      </c>
-      <c r="B5">
-        <v>63</v>
-      </c>
-      <c r="C5" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B6">
-        <v>105</v>
+        <v>464</v>
       </c>
       <c r="C6" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7">
-        <v>211</v>
+        <v>275</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8">
-        <v>464</v>
-      </c>
-      <c r="C8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9">
-        <v>942</v>
-      </c>
-      <c r="C9" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10">
-        <v>275</v>
-      </c>
-      <c r="C10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11">
-        <v>360</v>
-      </c>
-      <c r="C11" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated fnsga and comp testing
</commit_message>
<xml_diff>
--- a/datasets.xlsx
+++ b/datasets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erinfortin/Documents/Dissertation - Feature Selection/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D1BB1DC-72BF-6341-9851-301CBBDECD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F40CBA-8675-C545-90A5-0C21BA001021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7480" yWindow="680" windowWidth="10020" windowHeight="17380" xr2:uid="{44673F34-DF5D-4845-98A3-3A36EA99668B}"/>
   </bookViews>
@@ -56,18 +56,12 @@
     <t>isolet</t>
   </si>
   <si>
-    <t>spambase</t>
-  </si>
-  <si>
     <t>lymphography</t>
   </si>
   <si>
     <t>regression</t>
   </si>
   <si>
-    <t>bike-sharing</t>
-  </si>
-  <si>
     <t>wave-energy</t>
   </si>
   <si>
@@ -75,6 +69,12 @@
   </si>
   <si>
     <t>superconductivity</t>
+  </si>
+  <si>
+    <t>wine-quality</t>
+  </si>
+  <si>
+    <t>ionosphere</t>
   </si>
 </sst>
 </file>
@@ -473,10 +473,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B3">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="C3" t="s">
         <v>3</v>
@@ -484,7 +484,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4">
         <v>63</v>
@@ -495,35 +495,35 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B6">
         <v>464</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B7">
-        <v>275</v>
+        <v>186</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>